<commit_message>
does the most basic things - states the obvious with a greeting once you run it
</commit_message>
<xml_diff>
--- a/data/tracker.xlsx
+++ b/data/tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\14379\Desktop\uni\Fimbo\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E307EC95-B919-4384-B739-C9EC1975EE1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC273693-900A-4D90-9B18-5B24D74587C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DB9E5BB4-837A-42F7-A05C-7BDDFA2AA75B}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{DB9E5BB4-837A-42F7-A05C-7BDDFA2AA75B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Amount</t>
   </si>
@@ -50,10 +50,28 @@
     <t>Transaction Date</t>
   </si>
   <si>
-    <t>Transaction type</t>
-  </si>
-  <si>
-    <t>Cumulative Total</t>
+    <t>Debit</t>
+  </si>
+  <si>
+    <t>Credit</t>
+  </si>
+  <si>
+    <t>Cash</t>
+  </si>
+  <si>
+    <t>Food</t>
+  </si>
+  <si>
+    <t>Transport</t>
+  </si>
+  <si>
+    <t>Shopping</t>
+  </si>
+  <si>
+    <t>Transaction Type</t>
+  </si>
+  <si>
+    <t>Cumulative Amount</t>
   </si>
 </sst>
 </file>
@@ -97,9 +115,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -434,7 +460,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3EF4658-D9FA-4875-9DC2-6168826A0D0D}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="10" width="28" customWidth="1"/>
@@ -445,7 +471,7 @@
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -454,7 +480,58 @@
         <v>0</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="2">
+        <v>46143</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="3">
+        <v>15.5</v>
+      </c>
+      <c r="E2" s="3">
+        <v>15.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
+        <v>46143</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="E3" s="3">
+        <v>19.25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="2">
+        <v>46143</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>4</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="3">
+        <v>45</v>
+      </c>
+      <c r="E4" s="3">
+        <v>64.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
use streamlit to create initial working dashboard
</commit_message>
<xml_diff>
--- a/data/tracker.xlsx
+++ b/data/tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\14379\Desktop\uni\Fimbo\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC273693-900A-4D90-9B18-5B24D74587C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A21BB51-4646-40A2-A69A-8119B7960059}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{DB9E5BB4-837A-42F7-A05C-7BDDFA2AA75B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DB9E5BB4-837A-42F7-A05C-7BDDFA2AA75B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -502,7 +502,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>5</v>
@@ -519,7 +519,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
-        <v>46143</v>
+        <v>46145</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>4</v>

</xml_diff>

<commit_message>
add monthly trends and polish dashboard
</commit_message>
<xml_diff>
--- a/data/tracker.xlsx
+++ b/data/tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\14379\Desktop\uni\Fimbo\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A21BB51-4646-40A2-A69A-8119B7960059}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AED9F3AC-55EE-4D6B-BE19-B9D4B3CF756F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DB9E5BB4-837A-42F7-A05C-7BDDFA2AA75B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{DB9E5BB4-837A-42F7-A05C-7BDDFA2AA75B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
   <si>
     <t>Amount</t>
   </si>
@@ -115,16 +115,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -460,14 +466,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3EF4658-D9FA-4875-9DC2-6168826A0D0D}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="10" width="28" customWidth="1"/>
+    <col min="1" max="1" width="28" style="5" customWidth="1"/>
+    <col min="2" max="10" width="28" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -484,57 +491,101 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="2">
+      <c r="A2" s="4">
         <v>46143</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="2">
         <v>15.5</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="2">
+        <f>SUM($D$2:D2)</f>
         <v>15.5</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="2">
+      <c r="A3" s="4">
         <v>46144</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <v>3.75</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="2">
+        <f>SUM($D$2:D3)</f>
         <v>19.25</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="2">
+      <c r="A4" s="4">
         <v>46145</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <v>45</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="2">
+        <f>SUM($D$2:D4)</f>
         <v>64.25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="4">
+        <v>46177</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="2">
+        <v>5</v>
+      </c>
+      <c r="E5" s="2">
+        <f>SUM($D$2:D5)</f>
+        <v>69.25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="4">
+        <v>46211</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="2">
+        <v>50</v>
+      </c>
+      <c r="E6" s="2">
+        <f>SUM($D$2:D6)</f>
+        <v>119.25</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B1048576" xr:uid="{23AB770C-69E0-4A5A-BED6-A08589B3697F}">
+      <formula1>"Cash, Debit, Credit"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>